<commit_message>
fix: resolve redrob signals key name mismatch and regenerate correct candidate rankings
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -28,604 +28,604 @@
     <t>reasoning</t>
   </si>
   <si>
+    <t>CAND_0052328</t>
+  </si>
+  <si>
     <t>CAND_0046525</t>
   </si>
   <si>
+    <t>CAND_0065195</t>
+  </si>
+  <si>
+    <t>CAND_0027691</t>
+  </si>
+  <si>
+    <t>CAND_0098846</t>
+  </si>
+  <si>
+    <t>CAND_0086022</t>
+  </si>
+  <si>
     <t>CAND_0081852</t>
   </si>
   <si>
+    <t>CAND_0067866</t>
+  </si>
+  <si>
+    <t>CAND_0011687</t>
+  </si>
+  <si>
+    <t>CAND_0066999</t>
+  </si>
+  <si>
     <t>CAND_0045250</t>
   </si>
   <si>
-    <t>CAND_0052328</t>
+    <t>CAND_0041610</t>
+  </si>
+  <si>
+    <t>CAND_0081846</t>
   </si>
   <si>
     <t>CAND_0080766</t>
   </si>
   <si>
-    <t>CAND_0041610</t>
-  </si>
-  <si>
     <t>CAND_0095528</t>
   </si>
   <si>
-    <t>CAND_0098846</t>
-  </si>
-  <si>
-    <t>CAND_0081086</t>
-  </si>
-  <si>
-    <t>CAND_0065195</t>
+    <t>CAND_0018499</t>
+  </si>
+  <si>
+    <t>CAND_0052682</t>
+  </si>
+  <si>
+    <t>CAND_0079387</t>
+  </si>
+  <si>
+    <t>CAND_0046064</t>
+  </si>
+  <si>
+    <t>CAND_0058688</t>
+  </si>
+  <si>
+    <t>CAND_0075249</t>
+  </si>
+  <si>
+    <t>CAND_0041669</t>
+  </si>
+  <si>
+    <t>CAND_0073007</t>
+  </si>
+  <si>
+    <t>CAND_0074735</t>
+  </si>
+  <si>
+    <t>CAND_0077337</t>
+  </si>
+  <si>
+    <t>CAND_0055992</t>
   </si>
   <si>
     <t>CAND_0068811</t>
   </si>
   <si>
-    <t>CAND_0027691</t>
+    <t>CAND_0039754</t>
+  </si>
+  <si>
+    <t>CAND_0081053</t>
+  </si>
+  <si>
+    <t>CAND_0029971</t>
+  </si>
+  <si>
+    <t>CAND_0005649</t>
+  </si>
+  <si>
+    <t>CAND_0006418</t>
+  </si>
+  <si>
+    <t>CAND_0037160</t>
+  </si>
+  <si>
+    <t>CAND_0088025</t>
+  </si>
+  <si>
+    <t>CAND_0081480</t>
+  </si>
+  <si>
+    <t>CAND_0014063</t>
+  </si>
+  <si>
+    <t>CAND_0037566</t>
+  </si>
+  <si>
+    <t>CAND_0005260</t>
+  </si>
+  <si>
+    <t>CAND_0027801</t>
+  </si>
+  <si>
+    <t>CAND_0058575</t>
+  </si>
+  <si>
+    <t>CAND_0030348</t>
+  </si>
+  <si>
+    <t>CAND_0064326</t>
+  </si>
+  <si>
+    <t>CAND_0098454</t>
+  </si>
+  <si>
+    <t>CAND_0002025</t>
+  </si>
+  <si>
+    <t>CAND_0064888</t>
+  </si>
+  <si>
+    <t>CAND_0044883</t>
+  </si>
+  <si>
+    <t>CAND_0009024</t>
+  </si>
+  <si>
+    <t>CAND_0015528</t>
+  </si>
+  <si>
+    <t>CAND_0018549</t>
+  </si>
+  <si>
+    <t>CAND_0043860</t>
+  </si>
+  <si>
+    <t>CAND_0072688</t>
+  </si>
+  <si>
+    <t>CAND_0061257</t>
+  </si>
+  <si>
+    <t>CAND_0092839</t>
+  </si>
+  <si>
+    <t>CAND_0048558</t>
+  </si>
+  <si>
+    <t>CAND_0054394</t>
+  </si>
+  <si>
+    <t>CAND_0017960</t>
+  </si>
+  <si>
+    <t>CAND_0082973</t>
+  </si>
+  <si>
+    <t>CAND_0094728</t>
+  </si>
+  <si>
+    <t>CAND_0014440</t>
+  </si>
+  <si>
+    <t>CAND_0042029</t>
+  </si>
+  <si>
+    <t>CAND_0076251</t>
+  </si>
+  <si>
+    <t>CAND_0030031</t>
+  </si>
+  <si>
+    <t>CAND_0019880</t>
+  </si>
+  <si>
+    <t>CAND_0020350</t>
+  </si>
+  <si>
+    <t>CAND_0077498</t>
+  </si>
+  <si>
+    <t>CAND_0052335</t>
+  </si>
+  <si>
+    <t>CAND_0071974</t>
+  </si>
+  <si>
+    <t>CAND_0057563</t>
+  </si>
+  <si>
+    <t>CAND_0006557</t>
+  </si>
+  <si>
+    <t>CAND_0096142</t>
+  </si>
+  <si>
+    <t>CAND_0078492</t>
   </si>
   <si>
     <t>CAND_0046924</t>
   </si>
   <si>
-    <t>CAND_0086022</t>
-  </si>
-  <si>
-    <t>CAND_0027801</t>
-  </si>
-  <si>
-    <t>CAND_0067866</t>
-  </si>
-  <si>
-    <t>CAND_0099401</t>
-  </si>
-  <si>
-    <t>CAND_0074735</t>
-  </si>
-  <si>
-    <t>CAND_0005649</t>
-  </si>
-  <si>
-    <t>CAND_0005260</t>
-  </si>
-  <si>
-    <t>CAND_0044883</t>
-  </si>
-  <si>
-    <t>CAND_0082973</t>
+    <t>CAND_0061265</t>
   </si>
   <si>
     <t>CAND_0089947</t>
   </si>
   <si>
-    <t>CAND_0081053</t>
-  </si>
-  <si>
-    <t>CAND_0015528</t>
-  </si>
-  <si>
-    <t>CAND_0038368</t>
-  </si>
-  <si>
-    <t>CAND_0011687</t>
-  </si>
-  <si>
-    <t>CAND_0066999</t>
+    <t>CAND_0091534</t>
+  </si>
+  <si>
+    <t>CAND_0051292</t>
+  </si>
+  <si>
+    <t>CAND_0068351</t>
+  </si>
+  <si>
+    <t>CAND_0011162</t>
+  </si>
+  <si>
+    <t>CAND_0050876</t>
+  </si>
+  <si>
+    <t>CAND_0008295</t>
+  </si>
+  <si>
+    <t>CAND_0083879</t>
+  </si>
+  <si>
+    <t>CAND_0008425</t>
+  </si>
+  <si>
+    <t>CAND_0075439</t>
   </si>
   <si>
     <t>CAND_0049896</t>
   </si>
   <si>
-    <t>CAND_0047721</t>
-  </si>
-  <si>
-    <t>CAND_0006557</t>
-  </si>
-  <si>
-    <t>CAND_0081846</t>
-  </si>
-  <si>
-    <t>CAND_0087630</t>
-  </si>
-  <si>
-    <t>CAND_0075249</t>
-  </si>
-  <si>
-    <t>CAND_0088025</t>
-  </si>
-  <si>
-    <t>CAND_0094728</t>
-  </si>
-  <si>
-    <t>CAND_0031593</t>
-  </si>
-  <si>
-    <t>CAND_0011125</t>
-  </si>
-  <si>
-    <t>CAND_0010283</t>
-  </si>
-  <si>
-    <t>CAND_0058575</t>
-  </si>
-  <si>
-    <t>CAND_0018499</t>
-  </si>
-  <si>
-    <t>CAND_0052682</t>
-  </si>
-  <si>
-    <t>CAND_0079387</t>
-  </si>
-  <si>
-    <t>CAND_0041669</t>
-  </si>
-  <si>
-    <t>CAND_0040117</t>
-  </si>
-  <si>
-    <t>CAND_0046064</t>
-  </si>
-  <si>
-    <t>CAND_0064904</t>
-  </si>
-  <si>
-    <t>CAND_0073007</t>
-  </si>
-  <si>
-    <t>CAND_0096142</t>
-  </si>
-  <si>
-    <t>CAND_0030348</t>
-  </si>
-  <si>
-    <t>CAND_0058688</t>
-  </si>
-  <si>
-    <t>CAND_0091909</t>
-  </si>
-  <si>
-    <t>CAND_0029971</t>
-  </si>
-  <si>
-    <t>CAND_0077337</t>
-  </si>
-  <si>
-    <t>CAND_0061265</t>
-  </si>
-  <si>
-    <t>CAND_0055992</t>
-  </si>
-  <si>
-    <t>CAND_0010685</t>
-  </si>
-  <si>
-    <t>CAND_0009024</t>
-  </si>
-  <si>
-    <t>CAND_0057563</t>
-  </si>
-  <si>
-    <t>CAND_0070202</t>
-  </si>
-  <si>
-    <t>CAND_0010257</t>
-  </si>
-  <si>
-    <t>CAND_0006418</t>
-  </si>
-  <si>
-    <t>CAND_0044855</t>
-  </si>
-  <si>
-    <t>CAND_0031397</t>
-  </si>
-  <si>
-    <t>CAND_0094056</t>
-  </si>
-  <si>
-    <t>CAND_0011787</t>
-  </si>
-  <si>
-    <t>CAND_0079064</t>
-  </si>
-  <si>
-    <t>CAND_0086151</t>
-  </si>
-  <si>
-    <t>CAND_0096172</t>
+    <t>CAND_0077285</t>
+  </si>
+  <si>
+    <t>CAND_0073504</t>
+  </si>
+  <si>
+    <t>CAND_0073620</t>
+  </si>
+  <si>
+    <t>CAND_0015967</t>
+  </si>
+  <si>
+    <t>CAND_0010603</t>
   </si>
   <si>
     <t>CAND_0016163</t>
   </si>
   <si>
-    <t>CAND_0076251</t>
-  </si>
-  <si>
-    <t>CAND_0085851</t>
-  </si>
-  <si>
-    <t>CAND_0009691</t>
-  </si>
-  <si>
-    <t>CAND_0053934</t>
-  </si>
-  <si>
-    <t>CAND_0037566</t>
-  </si>
-  <si>
-    <t>CAND_0060835</t>
-  </si>
-  <si>
-    <t>CAND_0024466</t>
-  </si>
-  <si>
-    <t>CAND_0073620</t>
-  </si>
-  <si>
-    <t>CAND_0075439</t>
-  </si>
-  <si>
-    <t>CAND_0001056</t>
-  </si>
-  <si>
-    <t>CAND_0092712</t>
-  </si>
-  <si>
-    <t>CAND_0023093</t>
-  </si>
-  <si>
-    <t>CAND_0093547</t>
-  </si>
-  <si>
-    <t>CAND_0013393</t>
-  </si>
-  <si>
-    <t>CAND_0066179</t>
-  </si>
-  <si>
-    <t>CAND_0042029</t>
+    <t>CAND_0068932</t>
+  </si>
+  <si>
+    <t>CAND_0004402</t>
+  </si>
+  <si>
+    <t>CAND_0078002</t>
+  </si>
+  <si>
+    <t>CAND_0049538</t>
+  </si>
+  <si>
+    <t>CAND_0074486</t>
+  </si>
+  <si>
+    <t>CAND_0012397</t>
   </si>
   <si>
     <t>CAND_0030953</t>
   </si>
   <si>
-    <t>CAND_0032179</t>
-  </si>
-  <si>
-    <t>CAND_0066376</t>
-  </si>
-  <si>
-    <t>CAND_0088049</t>
-  </si>
-  <si>
-    <t>CAND_0030031</t>
-  </si>
-  <si>
-    <t>CAND_0011162</t>
-  </si>
-  <si>
-    <t>CAND_0089552</t>
-  </si>
-  <si>
-    <t>CAND_0071939</t>
-  </si>
-  <si>
-    <t>CAND_0008425</t>
-  </si>
-  <si>
-    <t>CAND_0098454</t>
-  </si>
-  <si>
-    <t>CAND_0060054</t>
-  </si>
-  <si>
-    <t>CAND_0039754</t>
-  </si>
-  <si>
-    <t>CAND_0081480</t>
-  </si>
-  <si>
-    <t>CAND_0012957</t>
-  </si>
-  <si>
-    <t>6yr Senior Machine Learning Engineer with production embedding/retrieval systems; 30d notice.</t>
-  </si>
-  <si>
-    <t>5yr Senior Data Scientist with production embedding/retrieval systems; 30d notice.</t>
-  </si>
-  <si>
-    <t>6yr Applied ML Engineer with production embedding/retrieval systems; 30d notice.</t>
-  </si>
-  <si>
-    <t>6yr Recommendation Systems Engineer with production embedding/retrieval systems; 30d notice.</t>
-  </si>
-  <si>
-    <t>8yr Staff Machine Learning Engineer with production embedding/retrieval systems; 30d notice.</t>
-  </si>
-  <si>
-    <t>6yr Recommendation Systems Engineer with production embedding/retrieval systems; 30d notice [CAND_0041610].</t>
-  </si>
-  <si>
-    <t>5yr Senior Data Scientist with production embedding/retrieval systems; 30d notice [CAND_0095528].</t>
-  </si>
-  <si>
-    <t>7yr AI Engineer with production embedding/retrieval systems; 30d notice.</t>
-  </si>
-  <si>
-    <t>5yr AI Specialist with production embedding/retrieval systems; low recent activity (flag).</t>
-  </si>
-  <si>
-    <t>5yr Search Engineer with production embedding/retrieval systems; 30d notice.</t>
+    <t>CAND_0018293</t>
+  </si>
+  <si>
+    <t>CAND_0013665</t>
+  </si>
+  <si>
+    <t>CAND_0097176</t>
+  </si>
+  <si>
+    <t>6yr Recommendation Systems Engineer with production embedding/retrieval systems; available immediately.</t>
+  </si>
+  <si>
+    <t>6yr Senior Machine Learning Engineer with production embedding/retrieval systems; 60d notice.</t>
+  </si>
+  <si>
+    <t>5yr Search Engineer with production embedding/retrieval systems; 45d notice.</t>
+  </si>
+  <si>
+    <t>6yr NLP Engineer with production embedding/retrieval systems; available immediately.</t>
+  </si>
+  <si>
+    <t>7yr AI Engineer with production embedding/retrieval systems; 45d notice.</t>
+  </si>
+  <si>
+    <t>5yr Senior Applied Scientist with production embedding/retrieval systems; available immediately.</t>
+  </si>
+  <si>
+    <t>5yr Senior Data Scientist with production embedding/retrieval systems; 45d notice.</t>
+  </si>
+  <si>
+    <t>6yr Senior Software Engineer (ML) with production embedding/retrieval systems; 45d notice.</t>
+  </si>
+  <si>
+    <t>7yr Senior NLP Engineer with production embedding/retrieval systems; available immediately.</t>
+  </si>
+  <si>
+    <t>5yr Recommendation Systems Engineer with production embedding/retrieval systems; available immediately.</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory.</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0041610].</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0081846].</t>
+  </si>
+  <si>
+    <t>8yr applied ML background; strong embeddings and vector DB match; solid career trajectory.</t>
+  </si>
+  <si>
+    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory.</t>
   </si>
   <si>
     <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory.</t>
   </si>
   <si>
-    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory.</t>
-  </si>
-  <si>
-    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0046924].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory.</t>
-  </si>
-  <si>
-    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0027801].</t>
-  </si>
-  <si>
-    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0067866].</t>
-  </si>
-  <si>
-    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0099401].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0074735].</t>
-  </si>
-  <si>
-    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0005649].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0005260].</t>
-  </si>
-  <si>
-    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0044883].</t>
-  </si>
-  <si>
-    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0082973].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0089947].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0081053].</t>
-  </si>
-  <si>
-    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0015528].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0038368].</t>
-  </si>
-  <si>
-    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0011687].</t>
-  </si>
-  <si>
-    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0066999].</t>
-  </si>
-  <si>
-    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0049896].</t>
-  </si>
-  <si>
-    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0047721].</t>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0052682].</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0079387].</t>
+  </si>
+  <si>
+    <t>8yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0046064].</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0058688].</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0075249].</t>
+  </si>
+  <si>
+    <t>7yr applied ML background; strong embeddings and vector DB match; noted short tenure history.</t>
+  </si>
+  <si>
+    <t>5yr applied ML background; strong embeddings and vector DB match; notice period 60d.</t>
+  </si>
+  <si>
+    <t>5yr applied ML background; strong embeddings and vector DB match; notice period 90d.</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; notice period 60d.</t>
+  </si>
+  <si>
+    <t>6yr applied ML background; strong embeddings and vector DB match; notice period 60d [CAND_0055992].</t>
+  </si>
+  <si>
+    <t>7yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0068811].</t>
+  </si>
+  <si>
+    <t>8yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0039754].</t>
+  </si>
+  <si>
+    <t>5yr applied ML background; strong embeddings and vector DB match; notice period 90d [CAND_0081053].</t>
+  </si>
+  <si>
+    <t>5yr applied ML background; strong embeddings and vector DB match; solid career trajectory [CAND_0029971].</t>
   </si>
   <si>
     <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience.</t>
   </si>
   <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0081846].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days.</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0075249].</t>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0006418].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0037160].</t>
   </si>
   <si>
     <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0088025].</t>
   </si>
   <si>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience.</t>
+  </si>
+  <si>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience [CAND_0014063].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: no production ML deployment found.</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0005260].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0027801].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0058575].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0030348].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: no production ML deployment found [CAND_0064326].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0098454].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0002025].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0064888].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: based outside India.</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0009024].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0015528].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0018549].</t>
+  </si>
+  <si>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience [CAND_0043860].</t>
+  </si>
+  <si>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience [CAND_0072688].</t>
+  </si>
+  <si>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience [CAND_0061257].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: no production ML deployment found [CAND_0092839].</t>
+  </si>
+  <si>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience [CAND_0048558].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: no production ML deployment found [CAND_0054394].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: no production ML deployment found [CAND_0017960].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0082973].</t>
+  </si>
+  <si>
     <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0094728].</t>
   </si>
   <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days [CAND_0031593].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days [CAND_0011125].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0010283].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0058575].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0018499].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0052682].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0079387].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0041669].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days [CAND_0040117].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0046064].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days [CAND_0064904].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0073007].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0096142].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0030348].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: based outside India.</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days [CAND_0091909].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0029971].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0077337].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0061265].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: based outside India [CAND_0055992].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: inactive &gt;90 days [CAND_0010685].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0009024].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0057563].</t>
-  </si>
-  <si>
-    <t>Partial fit — embedding systems understanding; concern: limited retrieval/ranking experience [CAND_0070202].</t>
+    <t>Partial fit — basic AI/ML skills; concern: limited retrieval/ranking experience [CAND_0014440].</t>
+  </si>
+  <si>
+    <t>Partial fit — embedding systems understanding; concern: no production ML deployment found [CAND_0042029].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements.</t>
   </si>
   <si>
     <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements.</t>
   </si>
   <si>
-    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0006418].</t>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0019880].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0020350].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements.</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0052335].</t>
   </si>
   <si>
     <t>Adjacent skills only — 7 relevant skills; low overall fit to requirements.</t>
   </si>
   <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements.</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 7 relevant skills; low overall fit to requirements [CAND_0094056].</t>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0057563].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 7 relevant skills; low overall fit to requirements [CAND_0006557].</t>
   </si>
   <si>
     <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements.</t>
   </si>
   <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0079064].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0086151].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0096172].</t>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0078492].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0046924].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0061265].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0089947].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0091534].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0051292].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0068351].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 9 relevant skills; low overall fit to requirements.</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 9 relevant skills; low overall fit to requirements [CAND_0050876].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 2 relevant skills; low overall fit to requirements.</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0083879].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0008425].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0075439].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0049896].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0077285].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 2 relevant skills; low overall fit to requirements [CAND_0073504].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0073620].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0015967].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0010603].</t>
   </si>
   <si>
     <t>Adjacent skills only — 7 relevant skills; low overall fit to requirements [CAND_0016163].</t>
   </si>
   <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0076251].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0085851].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0009691].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements.</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0037566].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 7 relevant skills; low overall fit to requirements [CAND_0060835].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0024466].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0073620].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0075439].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0001056].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0092712].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 2 relevant skills; low overall fit to requirements.</t>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0068932].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0004402].</t>
   </si>
   <si>
     <t>Adjacent skills only — 8 relevant skills; low overall fit to requirements.</t>
   </si>
   <si>
-    <t>Adjacent skills only — 8 relevant skills; low overall fit to requirements [CAND_0013393].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0066179].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 8 relevant skills; low overall fit to requirements [CAND_0042029].</t>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0049538].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0074486].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0012397].</t>
   </si>
   <si>
     <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0030953].</t>
   </si>
   <si>
-    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0032179].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0066376].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 2 relevant skills; low overall fit to requirements [CAND_0088049].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0030031].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 9 relevant skills; low overall fit to requirements.</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 7 relevant skills; low overall fit to requirements [CAND_0089552].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0071939].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 6 relevant skills; low overall fit to requirements [CAND_0008425].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0098454].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 4 relevant skills; low overall fit to requirements [CAND_0060054].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 9 relevant skills; low overall fit to requirements [CAND_0039754].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 2 relevant skills; low overall fit to requirements [CAND_0081480].</t>
-  </si>
-  <si>
-    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0012957].</t>
+    <t>Adjacent skills only — 3 relevant skills; low overall fit to requirements [CAND_0018293].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 5 relevant skills; low overall fit to requirements [CAND_0013665].</t>
+  </si>
+  <si>
+    <t>Adjacent skills only — 2 relevant skills; low overall fit to requirements [CAND_0097176].</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1008,7 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.615</v>
+        <v>0.7509</v>
       </c>
       <c r="D2" t="s">
         <v>104</v>
@@ -1022,7 +1022,7 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.6125</v>
+        <v>0.74</v>
       </c>
       <c r="D3" t="s">
         <v>105</v>
@@ -1036,7 +1036,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>0.6019</v>
+        <v>0.73</v>
       </c>
       <c r="D4" t="s">
         <v>106</v>
@@ -1050,7 +1050,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>0.6009</v>
+        <v>0.7274</v>
       </c>
       <c r="D5" t="s">
         <v>107</v>
@@ -1064,7 +1064,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>0.5971</v>
+        <v>0.724</v>
       </c>
       <c r="D6" t="s">
         <v>108</v>
@@ -1078,7 +1078,7 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>0.5873</v>
+        <v>0.7128</v>
       </c>
       <c r="D7" t="s">
         <v>109</v>
@@ -1092,7 +1092,7 @@
         <v>7</v>
       </c>
       <c r="C8">
-        <v>0.5864</v>
+        <v>0.7123</v>
       </c>
       <c r="D8" t="s">
         <v>110</v>
@@ -1106,7 +1106,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>0.5834</v>
+        <v>0.7113</v>
       </c>
       <c r="D9" t="s">
         <v>111</v>
@@ -1120,7 +1120,7 @@
         <v>9</v>
       </c>
       <c r="C10">
-        <v>0.5831</v>
+        <v>0.7086</v>
       </c>
       <c r="D10" t="s">
         <v>112</v>
@@ -1134,7 +1134,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.58</v>
+        <v>0.7085</v>
       </c>
       <c r="D11" t="s">
         <v>113</v>
@@ -1148,7 +1148,7 @@
         <v>11</v>
       </c>
       <c r="C12">
-        <v>0.578</v>
+        <v>0.7069</v>
       </c>
       <c r="D12" t="s">
         <v>114</v>
@@ -1162,7 +1162,7 @@
         <v>12</v>
       </c>
       <c r="C13">
-        <v>0.5774</v>
+        <v>0.7043</v>
       </c>
       <c r="D13" t="s">
         <v>115</v>
@@ -1176,7 +1176,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>0.577</v>
+        <v>0.7042</v>
       </c>
       <c r="D14" t="s">
         <v>116</v>
@@ -1190,7 +1190,7 @@
         <v>14</v>
       </c>
       <c r="C15">
-        <v>0.5767</v>
+        <v>0.701</v>
       </c>
       <c r="D15" t="s">
         <v>117</v>
@@ -1204,7 +1204,7 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>0.5746</v>
+        <v>0.6998</v>
       </c>
       <c r="D16" t="s">
         <v>118</v>
@@ -1218,7 +1218,7 @@
         <v>16</v>
       </c>
       <c r="C17">
-        <v>0.5738</v>
+        <v>0.6985</v>
       </c>
       <c r="D17" t="s">
         <v>119</v>
@@ -1232,7 +1232,7 @@
         <v>17</v>
       </c>
       <c r="C18">
-        <v>0.5714</v>
+        <v>0.6978</v>
       </c>
       <c r="D18" t="s">
         <v>120</v>
@@ -1246,7 +1246,7 @@
         <v>18</v>
       </c>
       <c r="C19">
-        <v>0.5712</v>
+        <v>0.6964</v>
       </c>
       <c r="D19" t="s">
         <v>121</v>
@@ -1260,7 +1260,7 @@
         <v>19</v>
       </c>
       <c r="C20">
-        <v>0.5701000000000001</v>
+        <v>0.695</v>
       </c>
       <c r="D20" t="s">
         <v>122</v>
@@ -1274,7 +1274,7 @@
         <v>20</v>
       </c>
       <c r="C21">
-        <v>0.5684</v>
+        <v>0.6934</v>
       </c>
       <c r="D21" t="s">
         <v>123</v>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C22">
-        <v>0.5676</v>
+        <v>0.6908</v>
       </c>
       <c r="D22" t="s">
         <v>124</v>
@@ -1302,7 +1302,7 @@
         <v>22</v>
       </c>
       <c r="C23">
-        <v>0.5639</v>
+        <v>0.6838</v>
       </c>
       <c r="D23" t="s">
         <v>125</v>
@@ -1316,7 +1316,7 @@
         <v>23</v>
       </c>
       <c r="C24">
-        <v>0.5627</v>
+        <v>0.6815</v>
       </c>
       <c r="D24" t="s">
         <v>126</v>
@@ -1330,7 +1330,7 @@
         <v>24</v>
       </c>
       <c r="C25">
-        <v>0.5615</v>
+        <v>0.6812</v>
       </c>
       <c r="D25" t="s">
         <v>127</v>
@@ -1344,7 +1344,7 @@
         <v>25</v>
       </c>
       <c r="C26">
-        <v>0.5602</v>
+        <v>0.6806</v>
       </c>
       <c r="D26" t="s">
         <v>128</v>
@@ -1358,7 +1358,7 @@
         <v>26</v>
       </c>
       <c r="C27">
-        <v>0.5588</v>
+        <v>0.6797</v>
       </c>
       <c r="D27" t="s">
         <v>129</v>
@@ -1372,7 +1372,7 @@
         <v>27</v>
       </c>
       <c r="C28">
-        <v>0.5586</v>
+        <v>0.6725</v>
       </c>
       <c r="D28" t="s">
         <v>130</v>
@@ -1386,7 +1386,7 @@
         <v>28</v>
       </c>
       <c r="C29">
-        <v>0.5585</v>
+        <v>0.6715</v>
       </c>
       <c r="D29" t="s">
         <v>131</v>
@@ -1400,7 +1400,7 @@
         <v>29</v>
       </c>
       <c r="C30">
-        <v>0.5563</v>
+        <v>0.6715</v>
       </c>
       <c r="D30" t="s">
         <v>132</v>
@@ -1414,7 +1414,7 @@
         <v>30</v>
       </c>
       <c r="C31">
-        <v>0.5561</v>
+        <v>0.669</v>
       </c>
       <c r="D31" t="s">
         <v>133</v>
@@ -1428,7 +1428,7 @@
         <v>31</v>
       </c>
       <c r="C32">
-        <v>0.5557</v>
+        <v>0.6641</v>
       </c>
       <c r="D32" t="s">
         <v>134</v>
@@ -1442,7 +1442,7 @@
         <v>32</v>
       </c>
       <c r="C33">
-        <v>0.5542</v>
+        <v>0.664</v>
       </c>
       <c r="D33" t="s">
         <v>135</v>
@@ -1456,7 +1456,7 @@
         <v>33</v>
       </c>
       <c r="C34">
-        <v>0.5534</v>
+        <v>0.6639</v>
       </c>
       <c r="D34" t="s">
         <v>136</v>
@@ -1470,7 +1470,7 @@
         <v>34</v>
       </c>
       <c r="C35">
-        <v>0.5533</v>
+        <v>0.6624</v>
       </c>
       <c r="D35" t="s">
         <v>137</v>
@@ -1484,7 +1484,7 @@
         <v>35</v>
       </c>
       <c r="C36">
-        <v>0.5524</v>
+        <v>0.659</v>
       </c>
       <c r="D36" t="s">
         <v>138</v>
@@ -1498,7 +1498,7 @@
         <v>36</v>
       </c>
       <c r="C37">
-        <v>0.5511</v>
+        <v>0.6564</v>
       </c>
       <c r="D37" t="s">
         <v>139</v>
@@ -1512,7 +1512,7 @@
         <v>37</v>
       </c>
       <c r="C38">
-        <v>0.5508999999999999</v>
+        <v>0.6561</v>
       </c>
       <c r="D38" t="s">
         <v>140</v>
@@ -1526,7 +1526,7 @@
         <v>38</v>
       </c>
       <c r="C39">
-        <v>0.5499000000000001</v>
+        <v>0.6559</v>
       </c>
       <c r="D39" t="s">
         <v>141</v>
@@ -1540,7 +1540,7 @@
         <v>39</v>
       </c>
       <c r="C40">
-        <v>0.5495</v>
+        <v>0.6551</v>
       </c>
       <c r="D40" t="s">
         <v>142</v>
@@ -1554,7 +1554,7 @@
         <v>40</v>
       </c>
       <c r="C41">
-        <v>0.5493</v>
+        <v>0.6493</v>
       </c>
       <c r="D41" t="s">
         <v>143</v>
@@ -1568,7 +1568,7 @@
         <v>41</v>
       </c>
       <c r="C42">
-        <v>0.5485</v>
+        <v>0.6492</v>
       </c>
       <c r="D42" t="s">
         <v>144</v>
@@ -1582,7 +1582,7 @@
         <v>42</v>
       </c>
       <c r="C43">
-        <v>0.5478</v>
+        <v>0.6483</v>
       </c>
       <c r="D43" t="s">
         <v>145</v>
@@ -1596,7 +1596,7 @@
         <v>43</v>
       </c>
       <c r="C44">
-        <v>0.5464</v>
+        <v>0.6468</v>
       </c>
       <c r="D44" t="s">
         <v>146</v>
@@ -1610,7 +1610,7 @@
         <v>44</v>
       </c>
       <c r="C45">
-        <v>0.5463</v>
+        <v>0.6467000000000001</v>
       </c>
       <c r="D45" t="s">
         <v>147</v>
@@ -1624,7 +1624,7 @@
         <v>45</v>
       </c>
       <c r="C46">
-        <v>0.5459000000000001</v>
+        <v>0.6466</v>
       </c>
       <c r="D46" t="s">
         <v>148</v>
@@ -1638,7 +1638,7 @@
         <v>46</v>
       </c>
       <c r="C47">
-        <v>0.545</v>
+        <v>0.6446</v>
       </c>
       <c r="D47" t="s">
         <v>149</v>
@@ -1652,7 +1652,7 @@
         <v>47</v>
       </c>
       <c r="C48">
-        <v>0.545</v>
+        <v>0.644</v>
       </c>
       <c r="D48" t="s">
         <v>150</v>
@@ -1666,7 +1666,7 @@
         <v>48</v>
       </c>
       <c r="C49">
-        <v>0.544</v>
+        <v>0.6435999999999999</v>
       </c>
       <c r="D49" t="s">
         <v>151</v>
@@ -1680,7 +1680,7 @@
         <v>49</v>
       </c>
       <c r="C50">
-        <v>0.544</v>
+        <v>0.642</v>
       </c>
       <c r="D50" t="s">
         <v>152</v>
@@ -1694,7 +1694,7 @@
         <v>50</v>
       </c>
       <c r="C51">
-        <v>0.5434</v>
+        <v>0.6408</v>
       </c>
       <c r="D51" t="s">
         <v>153</v>
@@ -1708,7 +1708,7 @@
         <v>51</v>
       </c>
       <c r="C52">
-        <v>0.5434</v>
+        <v>0.6385999999999999</v>
       </c>
       <c r="D52" t="s">
         <v>154</v>
@@ -1722,7 +1722,7 @@
         <v>52</v>
       </c>
       <c r="C53">
-        <v>0.5434</v>
+        <v>0.638</v>
       </c>
       <c r="D53" t="s">
         <v>155</v>
@@ -1736,7 +1736,7 @@
         <v>53</v>
       </c>
       <c r="C54">
-        <v>0.5431</v>
+        <v>0.6378</v>
       </c>
       <c r="D54" t="s">
         <v>156</v>
@@ -1750,7 +1750,7 @@
         <v>54</v>
       </c>
       <c r="C55">
-        <v>0.5431</v>
+        <v>0.6365</v>
       </c>
       <c r="D55" t="s">
         <v>157</v>
@@ -1764,7 +1764,7 @@
         <v>55</v>
       </c>
       <c r="C56">
-        <v>0.5425</v>
+        <v>0.6349</v>
       </c>
       <c r="D56" t="s">
         <v>158</v>
@@ -1778,7 +1778,7 @@
         <v>56</v>
       </c>
       <c r="C57">
-        <v>0.5422</v>
+        <v>0.6348</v>
       </c>
       <c r="D57" t="s">
         <v>159</v>
@@ -1792,7 +1792,7 @@
         <v>57</v>
       </c>
       <c r="C58">
-        <v>0.5407999999999999</v>
+        <v>0.6348</v>
       </c>
       <c r="D58" t="s">
         <v>160</v>
@@ -1806,7 +1806,7 @@
         <v>58</v>
       </c>
       <c r="C59">
-        <v>0.5405</v>
+        <v>0.6343</v>
       </c>
       <c r="D59" t="s">
         <v>161</v>
@@ -1820,7 +1820,7 @@
         <v>59</v>
       </c>
       <c r="C60">
-        <v>0.5399</v>
+        <v>0.6325</v>
       </c>
       <c r="D60" t="s">
         <v>162</v>
@@ -1834,7 +1834,7 @@
         <v>60</v>
       </c>
       <c r="C61">
-        <v>0.5397999999999999</v>
+        <v>0.6317</v>
       </c>
       <c r="D61" t="s">
         <v>163</v>
@@ -1848,7 +1848,7 @@
         <v>61</v>
       </c>
       <c r="C62">
-        <v>0.5394</v>
+        <v>0.6302</v>
       </c>
       <c r="D62" t="s">
         <v>164</v>
@@ -1862,7 +1862,7 @@
         <v>62</v>
       </c>
       <c r="C63">
-        <v>0.539</v>
+        <v>0.6292</v>
       </c>
       <c r="D63" t="s">
         <v>165</v>
@@ -1876,7 +1876,7 @@
         <v>63</v>
       </c>
       <c r="C64">
-        <v>0.539</v>
+        <v>0.6279</v>
       </c>
       <c r="D64" t="s">
         <v>166</v>
@@ -1890,7 +1890,7 @@
         <v>64</v>
       </c>
       <c r="C65">
-        <v>0.5387</v>
+        <v>0.6279</v>
       </c>
       <c r="D65" t="s">
         <v>167</v>
@@ -1904,7 +1904,7 @@
         <v>65</v>
       </c>
       <c r="C66">
-        <v>0.5379</v>
+        <v>0.6279</v>
       </c>
       <c r="D66" t="s">
         <v>168</v>
@@ -1918,7 +1918,7 @@
         <v>66</v>
       </c>
       <c r="C67">
-        <v>0.5376</v>
+        <v>0.6278</v>
       </c>
       <c r="D67" t="s">
         <v>169</v>
@@ -1932,7 +1932,7 @@
         <v>67</v>
       </c>
       <c r="C68">
-        <v>0.5376</v>
+        <v>0.6277</v>
       </c>
       <c r="D68" t="s">
         <v>170</v>
@@ -1946,7 +1946,7 @@
         <v>68</v>
       </c>
       <c r="C69">
-        <v>0.5371</v>
+        <v>0.6274</v>
       </c>
       <c r="D69" t="s">
         <v>171</v>
@@ -1960,7 +1960,7 @@
         <v>69</v>
       </c>
       <c r="C70">
-        <v>0.5368000000000001</v>
+        <v>0.6266</v>
       </c>
       <c r="D70" t="s">
         <v>172</v>
@@ -1974,7 +1974,7 @@
         <v>70</v>
       </c>
       <c r="C71">
-        <v>0.5363</v>
+        <v>0.6264999999999999</v>
       </c>
       <c r="D71" t="s">
         <v>173</v>
@@ -1988,7 +1988,7 @@
         <v>71</v>
       </c>
       <c r="C72">
-        <v>0.5346</v>
+        <v>0.6252</v>
       </c>
       <c r="D72" t="s">
         <v>174</v>
@@ -2002,7 +2002,7 @@
         <v>72</v>
       </c>
       <c r="C73">
-        <v>0.5346</v>
+        <v>0.625</v>
       </c>
       <c r="D73" t="s">
         <v>175</v>
@@ -2016,7 +2016,7 @@
         <v>73</v>
       </c>
       <c r="C74">
-        <v>0.5334</v>
+        <v>0.625</v>
       </c>
       <c r="D74" t="s">
         <v>176</v>
@@ -2030,7 +2030,7 @@
         <v>74</v>
       </c>
       <c r="C75">
-        <v>0.5329</v>
+        <v>0.6247</v>
       </c>
       <c r="D75" t="s">
         <v>177</v>
@@ -2044,7 +2044,7 @@
         <v>75</v>
       </c>
       <c r="C76">
-        <v>0.5324</v>
+        <v>0.6245000000000001</v>
       </c>
       <c r="D76" t="s">
         <v>178</v>
@@ -2058,7 +2058,7 @@
         <v>76</v>
       </c>
       <c r="C77">
-        <v>0.5321</v>
+        <v>0.6243</v>
       </c>
       <c r="D77" t="s">
         <v>179</v>
@@ -2072,7 +2072,7 @@
         <v>77</v>
       </c>
       <c r="C78">
-        <v>0.5308</v>
+        <v>0.6239</v>
       </c>
       <c r="D78" t="s">
         <v>180</v>
@@ -2086,7 +2086,7 @@
         <v>78</v>
       </c>
       <c r="C79">
-        <v>0.5302</v>
+        <v>0.6229</v>
       </c>
       <c r="D79" t="s">
         <v>181</v>
@@ -2100,7 +2100,7 @@
         <v>79</v>
       </c>
       <c r="C80">
-        <v>0.529</v>
+        <v>0.6228</v>
       </c>
       <c r="D80" t="s">
         <v>182</v>
@@ -2114,7 +2114,7 @@
         <v>80</v>
       </c>
       <c r="C81">
-        <v>0.5288</v>
+        <v>0.6218</v>
       </c>
       <c r="D81" t="s">
         <v>183</v>
@@ -2128,7 +2128,7 @@
         <v>81</v>
       </c>
       <c r="C82">
-        <v>0.528</v>
+        <v>0.6216</v>
       </c>
       <c r="D82" t="s">
         <v>184</v>
@@ -2142,7 +2142,7 @@
         <v>82</v>
       </c>
       <c r="C83">
-        <v>0.5278</v>
+        <v>0.6215000000000001</v>
       </c>
       <c r="D83" t="s">
         <v>185</v>
@@ -2156,7 +2156,7 @@
         <v>83</v>
       </c>
       <c r="C84">
-        <v>0.5272</v>
+        <v>0.6211</v>
       </c>
       <c r="D84" t="s">
         <v>186</v>
@@ -2170,7 +2170,7 @@
         <v>84</v>
       </c>
       <c r="C85">
-        <v>0.5265</v>
+        <v>0.6208</v>
       </c>
       <c r="D85" t="s">
         <v>187</v>
@@ -2184,7 +2184,7 @@
         <v>85</v>
       </c>
       <c r="C86">
-        <v>0.526</v>
+        <v>0.6207</v>
       </c>
       <c r="D86" t="s">
         <v>188</v>
@@ -2198,7 +2198,7 @@
         <v>86</v>
       </c>
       <c r="C87">
-        <v>0.5259</v>
+        <v>0.6204</v>
       </c>
       <c r="D87" t="s">
         <v>189</v>
@@ -2212,7 +2212,7 @@
         <v>87</v>
       </c>
       <c r="C88">
-        <v>0.5254</v>
+        <v>0.6199</v>
       </c>
       <c r="D88" t="s">
         <v>190</v>
@@ -2226,7 +2226,7 @@
         <v>88</v>
       </c>
       <c r="C89">
-        <v>0.5252</v>
+        <v>0.6198</v>
       </c>
       <c r="D89" t="s">
         <v>191</v>
@@ -2240,7 +2240,7 @@
         <v>89</v>
       </c>
       <c r="C90">
-        <v>0.5252</v>
+        <v>0.6191</v>
       </c>
       <c r="D90" t="s">
         <v>192</v>
@@ -2254,7 +2254,7 @@
         <v>90</v>
       </c>
       <c r="C91">
-        <v>0.5252</v>
+        <v>0.6188</v>
       </c>
       <c r="D91" t="s">
         <v>193</v>
@@ -2268,7 +2268,7 @@
         <v>91</v>
       </c>
       <c r="C92">
-        <v>0.5242</v>
+        <v>0.6188</v>
       </c>
       <c r="D92" t="s">
         <v>194</v>
@@ -2282,7 +2282,7 @@
         <v>92</v>
       </c>
       <c r="C93">
-        <v>0.5229</v>
+        <v>0.6187</v>
       </c>
       <c r="D93" t="s">
         <v>195</v>
@@ -2296,7 +2296,7 @@
         <v>93</v>
       </c>
       <c r="C94">
-        <v>0.5229</v>
+        <v>0.6183</v>
       </c>
       <c r="D94" t="s">
         <v>196</v>
@@ -2310,7 +2310,7 @@
         <v>94</v>
       </c>
       <c r="C95">
-        <v>0.5226</v>
+        <v>0.6173</v>
       </c>
       <c r="D95" t="s">
         <v>197</v>
@@ -2324,7 +2324,7 @@
         <v>95</v>
       </c>
       <c r="C96">
-        <v>0.5225</v>
+        <v>0.6168</v>
       </c>
       <c r="D96" t="s">
         <v>198</v>
@@ -2338,7 +2338,7 @@
         <v>96</v>
       </c>
       <c r="C97">
-        <v>0.5218</v>
+        <v>0.6163999999999999</v>
       </c>
       <c r="D97" t="s">
         <v>199</v>
@@ -2352,7 +2352,7 @@
         <v>97</v>
       </c>
       <c r="C98">
-        <v>0.5217000000000001</v>
+        <v>0.6163999999999999</v>
       </c>
       <c r="D98" t="s">
         <v>200</v>
@@ -2366,7 +2366,7 @@
         <v>98</v>
       </c>
       <c r="C99">
-        <v>0.5215</v>
+        <v>0.616</v>
       </c>
       <c r="D99" t="s">
         <v>201</v>
@@ -2380,7 +2380,7 @@
         <v>99</v>
       </c>
       <c r="C100">
-        <v>0.5215</v>
+        <v>0.6159</v>
       </c>
       <c r="D100" t="s">
         <v>202</v>
@@ -2394,7 +2394,7 @@
         <v>100</v>
       </c>
       <c r="C101">
-        <v>0.5211</v>
+        <v>0.6156</v>
       </c>
       <c r="D101" t="s">
         <v>203</v>

</xml_diff>